<commit_message>
TICVAI r2: the five BOCA document addresses Chinmay forwarded on 6 October, in the client source, ADR-0015 and the hardware workbook (CHG-R4-002)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ticvai/handoff/TICVAI_Hardware_Integration_annotated_v1_1.xlsx
+++ b/ticvai/handoff/TICVAI_Hardware_Integration_annotated_v1_1.xlsx
@@ -1010,7 +1010,12 @@
       </c>
       <c r="G15" s="16" t="inlineStr">
         <is>
-          <t>5 Oct 2026, Muhamed Allam: printer specifications; SDK sample codes; operator manuals and FGL programming guide; RFID encoding on the BOCA Lemur; Windows driver (link titles only, URLs pending; sources/client/2026-10-05-allam-boca-printer.md).</t>
+          <t>5 Oct 2026, Muhamed Allam: printer specifications; SDK sample codes; operator manuals and FGL programming guide; RFID encoding on the BOCA Lemur; Windows driver (sources/client/2026-10-05-allam-boca-printer.md).
+Specifications: https://tls-bocasystems.com/en/857/specifications/
+SDK sample code: https://tlsbocasystems.freshdesk.com/support/solutions/articles/62000051763-sample-code-and-sdk
+Operator manuals and programming guide: https://tlsbocasystems.freshdesk.com/support/solutions/articles/62000068126-operator-s-manuals-and-programming-guide
+RFID encoding on the Lemur: https://tlsbocasystems.freshdesk.com/support/solutions/articles/62000201858
+Windows driver: https://tlsbocasystems.freshdesk.com/support/solutions/articles/62000222844-windows-driver</t>
         </is>
       </c>
       <c r="H15" s="16" t="inlineStr">

</xml_diff>